<commit_message>
Reports completed only designing and alignment left
</commit_message>
<xml_diff>
--- a/public/reports/daily_pickup_sales_report.xlsx
+++ b/public/reports/daily_pickup_sales_report.xlsx
@@ -15,12 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="24">
   <si>
     <t>S. No.</t>
   </si>
   <si>
-    <t>Origin2018-08-15 00:00:00</t>
+    <t>Origin 2018-08-31</t>
   </si>
   <si>
     <t>No. of Parcels Booked</t>
@@ -65,7 +65,7 @@
     <t>Multan</t>
   </si>
   <si>
-    <t>DSR2018-08-15 00:00:00</t>
+    <t>DSR 2018-08-31</t>
   </si>
   <si>
     <t>Farrell Ltd</t>
@@ -84,6 +84,9 @@
   </si>
   <si>
     <t>Mohr-Collier</t>
+  </si>
+  <si>
+    <t>Torp, Stamm and Wilkinson</t>
   </si>
 </sst>
 </file>
@@ -434,8 +437,8 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
-  <sheetFormatPr defaultRowHeight="14.4" defaultColWidth="30" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr defaultRowHeight="14.4" defaultColWidth="20" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
@@ -462,260 +465,149 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="1">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="1">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="1">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="1">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="1">
+      <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="1">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8" s="1">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-    </row>
-    <row r="17" spans="1:9">
-      <c r="A17" s="1" t="s">
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="1" t="s">
+      <c r="G21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H21" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H17" s="1" t="s">
+      <c r="I21" s="1" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
-      <c r="A18">
-        <v>1</v>
-      </c>
-      <c r="B18" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
-      <c r="A19">
-        <v>2</v>
-      </c>
-      <c r="B19" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
-      <c r="A20">
-        <v>3</v>
-      </c>
-      <c r="B20" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21">
-        <v>4</v>
-      </c>
-      <c r="B21" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23">
+        <v>2</v>
+      </c>
+      <c r="B23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24">
+        <v>3</v>
+      </c>
+      <c r="B24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26">
+        <v>5</v>
+      </c>
+      <c r="B26" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27">
         <v>6</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B27" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28">
+        <v>7</v>
+      </c>
+      <c r="B28" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>